<commit_message>
Mejora de la arquitectura paquete config
Preparando práctica de pruebas unidad
Context se encarga de construir los objetos de consulta de métricas e
indicadores. Context es la única responsable del contexto de la API

Para las clases de consulta de métricas e indicadores se han creado por
separado el caso de fichero configurado por el cliente y no (test y
test2)
Se han separado en métodos de test individuales cada caso (se ha dejado
uno complejo en IndicadorTest para mostrar la diferencia)

Revisado RepositoryCalculatorTest
</commit_message>
<xml_diff>
--- a/src/test/resources/excelTest.xlsx
+++ b/src/test/resources/excelTest.xlsx
@@ -10,11 +10,11 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC655F3E-7AB5-4883-B9AE-5A0605A2270F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3675" yWindow="5415" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3675" yWindow="5415" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="entidadTest" r:id="rId5" sheetId="1"/>
     <sheet name="MIT-FS.Audit4Improve-API" r:id="rId6" sheetId="2"/>
+    <sheet name="entidadTest" r:id="rId5" sheetId="3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1034" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1068" uniqueCount="122">
   <si>
     <t xml:space="preserve">Métricas guardadas el día </t>
   </si>
@@ -383,6 +383,15 @@
   </si>
   <si>
     <t>Fri Mar 08 15:38:20 CET 2024</t>
+  </si>
+  <si>
+    <t>Mon Mar 17 11:10:14 CET 2025</t>
+  </si>
+  <si>
+    <t>Mon Mar 17 11:10:15 CET 2025</t>
+  </si>
+  <si>
+    <t>Mon Mar 17 10:10:15 CET 2025</t>
   </si>
 </sst>
 </file>
@@ -390,7 +399,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="24">
+  <fonts count="27">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -534,6 +543,24 @@
       <name val="Serif"/>
       <sz val="10.0"/>
       <color rgb="FF00FF00"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="15.0"/>
+      <color rgb="FFFF0000"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Courier New"/>
+      <sz val="20.0"/>
+      <color rgb="FFFF0000"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Serif"/>
+      <sz val="10.0"/>
+      <color rgb="FFFFC800"/>
       <b val="true"/>
     </font>
   </fonts>
@@ -572,7 +599,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -597,6 +624,9 @@
     <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
     <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -875,18 +905,17 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="21.9375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="24.55859375"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="9.703125"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="32.12109375"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="11.1328125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="25.796875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="11.52734375"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="51.4921875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="15.01171875"/>
     <col min="6" max="6" bestFit="true" customWidth="true" width="24.55859375"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="24.55859375"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -894,111 +923,292 @@
         <v>0</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>25</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="4">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s" s="4">
-        <v>3</v>
+      <c r="A2" t="s" s="23">
+        <v>28</v>
+      </c>
+      <c r="B2" t="s" s="23">
+        <v>29</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="E2" s="0"/>
+        <v>30</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>31</v>
+      </c>
       <c r="F2" t="s" s="0">
-        <v>26</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s" s="4">
+      <c r="A3" t="s" s="23">
+        <v>102</v>
+      </c>
+      <c r="B3" t="s" s="23">
+        <v>103</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>104</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="23">
+        <v>86</v>
+      </c>
+      <c r="B4" t="s" s="23">
+        <v>87</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>89</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="23">
+        <v>62</v>
+      </c>
+      <c r="B5" t="s" s="23">
+        <v>63</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>66</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="23">
+        <v>67</v>
+      </c>
+      <c r="B6" t="s" s="23">
+        <v>63</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>66</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="23">
+        <v>33</v>
+      </c>
+      <c r="B7" t="s" s="23">
+        <v>34</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="F7" t="s" s="0">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="23">
+        <v>36</v>
+      </c>
+      <c r="B8" t="s" s="23">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="F8" t="s" s="0">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="23">
+        <v>42</v>
+      </c>
+      <c r="B9" t="s" s="23">
+        <v>37</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="F9" t="s" s="0">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="23">
+        <v>44</v>
+      </c>
+      <c r="B10" t="s" s="23">
+        <v>98</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>99</v>
+      </c>
+      <c r="E10" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="F10" t="s" s="0">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="23">
+        <v>106</v>
+      </c>
+      <c r="B11" t="s" s="23">
+        <v>15</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="D11" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="E11" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="F11" t="s" s="0">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="23">
         <v>5</v>
       </c>
-      <c r="B3" t="s" s="4">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s" s="0">
+      <c r="B12" t="s" s="23">
+        <v>61</v>
+      </c>
+      <c r="C12" t="s" s="0">
         <v>7</v>
       </c>
-      <c r="D3" t="s" s="0">
+      <c r="D12" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="E3" s="0"/>
-      <c r="F3" t="s" s="0">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
+      <c r="E12" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="F12" t="s" s="0">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="23">
+        <v>51</v>
+      </c>
+      <c r="B13" t="s" s="23">
+        <v>52</v>
+      </c>
+      <c r="C13" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="D13" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="E13" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="F13" t="s" s="0">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="23">
+        <v>91</v>
+      </c>
+      <c r="B14" t="s" s="23">
+        <v>92</v>
+      </c>
+      <c r="C14" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="D14" t="s" s="0">
+        <v>93</v>
+      </c>
+      <c r="E14" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="F14" t="s" s="0">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="23">
+        <v>46</v>
+      </c>
+      <c r="B15" t="s" s="23">
+        <v>47</v>
+      </c>
+      <c r="C15" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="D15" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="E15" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="F15" t="s" s="0">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="0">
         <v>1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="5">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s" s="5">
-        <v>10</v>
-      </c>
-      <c r="C5" t="s" s="0">
-        <v>11</v>
-      </c>
-      <c r="D5" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" s="0"/>
-      <c r="G5" t="s" s="0">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="6">
-        <v>14</v>
-      </c>
-      <c r="B6" t="s" s="6">
-        <v>15</v>
-      </c>
-      <c r="C6" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="D6" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="F6" s="0"/>
-      <c r="G6" t="s" s="0">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s" s="5">
-        <v>19</v>
-      </c>
-      <c r="B7" t="s" s="5">
-        <v>20</v>
-      </c>
-      <c r="C7" t="s" s="0">
-        <v>21</v>
-      </c>
-      <c r="D7" t="s" s="0">
-        <v>22</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" s="0"/>
-      <c r="G7" t="s" s="0">
-        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -1006,17 +1216,18 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="21.9375" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="25.796875" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="11.52734375" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="51.4921875" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="15.01171875" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="24.55859375" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="23.38671875" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="26.27734375" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="9.703125" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="32.12109375" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="26.27734375" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="19.08203125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="26.27734375" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1024,292 +1235,111 @@
         <v>0</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="23">
-        <v>28</v>
-      </c>
-      <c r="B2" t="s" s="23">
-        <v>29</v>
+      <c r="A2" t="s" s="24">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s" s="24">
+        <v>3</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>30</v>
-      </c>
-      <c r="E2" t="s" s="0">
-        <v>31</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="E2" s="0"/>
       <c r="F2" t="s" s="0">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s" s="23">
-        <v>102</v>
-      </c>
-      <c r="B3" t="s" s="23">
-        <v>103</v>
+      <c r="A3" t="s" s="24">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s" s="24">
+        <v>6</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>44</v>
+        <v>7</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>104</v>
-      </c>
-      <c r="E3" t="s" s="0">
-        <v>31</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="E3" s="0"/>
       <c r="F3" t="s" s="0">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="s" s="23">
-        <v>86</v>
-      </c>
-      <c r="B4" t="s" s="23">
-        <v>87</v>
-      </c>
-      <c r="C4" t="s" s="0">
-        <v>88</v>
-      </c>
-      <c r="D4" t="s" s="0">
-        <v>89</v>
-      </c>
-      <c r="E4" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="F4" t="s" s="0">
-        <v>117</v>
+      <c r="A4" t="s" s="0">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="s" s="23">
-        <v>62</v>
-      </c>
-      <c r="B5" t="s" s="23">
-        <v>63</v>
+      <c r="A5" t="s" s="25">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s" s="25">
+        <v>10</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>64</v>
+        <v>11</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="E5" t="s" s="0">
-        <v>66</v>
-      </c>
-      <c r="F5" t="s" s="0">
-        <v>117</v>
+        <v>12</v>
+      </c>
+      <c r="E5" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="0"/>
+      <c r="G5" t="s" s="0">
+        <v>121</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="s" s="23">
-        <v>67</v>
-      </c>
-      <c r="B6" t="s" s="23">
-        <v>63</v>
+      <c r="A6" t="s" s="26">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s" s="26">
+        <v>15</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>68</v>
+        <v>16</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>69</v>
-      </c>
-      <c r="E6" t="s" s="0">
-        <v>66</v>
-      </c>
-      <c r="F6" t="s" s="0">
-        <v>117</v>
+        <v>17</v>
+      </c>
+      <c r="E6" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="0"/>
+      <c r="G6" t="s" s="0">
+        <v>121</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="s" s="23">
-        <v>33</v>
-      </c>
-      <c r="B7" t="s" s="23">
-        <v>34</v>
+      <c r="A7" t="s" s="25">
+        <v>19</v>
+      </c>
+      <c r="B7" t="s" s="25">
+        <v>20</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>35</v>
-      </c>
-      <c r="E7" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="F7" t="s" s="0">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s" s="23">
-        <v>36</v>
-      </c>
-      <c r="B8" t="s" s="23">
-        <v>37</v>
-      </c>
-      <c r="C8" t="s" s="0">
-        <v>36</v>
-      </c>
-      <c r="D8" t="s" s="0">
-        <v>38</v>
-      </c>
-      <c r="E8" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="F8" t="s" s="0">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s" s="23">
-        <v>42</v>
-      </c>
-      <c r="B9" t="s" s="23">
-        <v>37</v>
-      </c>
-      <c r="C9" t="s" s="0">
-        <v>42</v>
-      </c>
-      <c r="D9" t="s" s="0">
-        <v>43</v>
-      </c>
-      <c r="E9" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="F9" t="s" s="0">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s" s="23">
-        <v>44</v>
-      </c>
-      <c r="B10" t="s" s="23">
-        <v>98</v>
-      </c>
-      <c r="C10" t="s" s="0">
-        <v>44</v>
-      </c>
-      <c r="D10" t="s" s="0">
-        <v>99</v>
-      </c>
-      <c r="E10" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="F10" t="s" s="0">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s" s="23">
-        <v>106</v>
-      </c>
-      <c r="B11" t="s" s="23">
-        <v>15</v>
-      </c>
-      <c r="C11" t="s" s="0">
-        <v>44</v>
-      </c>
-      <c r="D11" t="s" s="0">
-        <v>45</v>
-      </c>
-      <c r="E11" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="F11" t="s" s="0">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s" s="23">
-        <v>5</v>
-      </c>
-      <c r="B12" t="s" s="23">
-        <v>61</v>
-      </c>
-      <c r="C12" t="s" s="0">
-        <v>7</v>
-      </c>
-      <c r="D12" t="s" s="0">
-        <v>8</v>
-      </c>
-      <c r="E12" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="F12" t="s" s="0">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s" s="23">
-        <v>51</v>
-      </c>
-      <c r="B13" t="s" s="23">
-        <v>52</v>
-      </c>
-      <c r="C13" t="s" s="0">
-        <v>7</v>
-      </c>
-      <c r="D13" t="s" s="0">
-        <v>53</v>
-      </c>
-      <c r="E13" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="F13" t="s" s="0">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s" s="23">
-        <v>91</v>
-      </c>
-      <c r="B14" t="s" s="23">
-        <v>92</v>
-      </c>
-      <c r="C14" t="s" s="0">
-        <v>91</v>
-      </c>
-      <c r="D14" t="s" s="0">
-        <v>93</v>
-      </c>
-      <c r="E14" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="F14" t="s" s="0">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="s" s="23">
-        <v>46</v>
-      </c>
-      <c r="B15" t="s" s="23">
-        <v>47</v>
-      </c>
-      <c r="C15" t="s" s="0">
-        <v>7</v>
-      </c>
-      <c r="D15" t="s" s="0">
-        <v>48</v>
-      </c>
-      <c r="E15" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="F15" t="s" s="0">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="s" s="0">
-        <v>1</v>
+        <v>22</v>
+      </c>
+      <c r="E7" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="0"/>
+      <c r="G7" t="s" s="0">
+        <v>121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Hecho el test para la métrica que mide el número de líneas escritas en el último mes
</commit_message>
<xml_diff>
--- a/src/test/resources/excelTest.xlsx
+++ b/src/test/resources/excelTest.xlsx
@@ -13,8 +13,8 @@
     <workbookView xWindow="3675" yWindow="5415" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="MIT-FS.Audit4Improve-API" r:id="rId6" sheetId="2"/>
     <sheet name="entidadTest" r:id="rId5" sheetId="3"/>
+    <sheet name="MIT-FS.Audit4Improve-API" r:id="rId6" sheetId="4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1068" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1111" uniqueCount="128">
   <si>
     <t xml:space="preserve">Métricas guardadas el día </t>
   </si>
@@ -392,6 +392,24 @@
   </si>
   <si>
     <t>Mon Mar 17 10:10:15 CET 2025</t>
+  </si>
+  <si>
+    <t>Fri May 30 20:14:41 CEST 2025</t>
+  </si>
+  <si>
+    <t>Fri May 30 20:14:42 CEST 2025</t>
+  </si>
+  <si>
+    <t>Fri May 30 18:14:42 CEST 2025</t>
+  </si>
+  <si>
+    <t>Fri May 30 20:14:44 CEST 2025</t>
+  </si>
+  <si>
+    <t>7010</t>
+  </si>
+  <si>
+    <t>Fri May 30 20:14:43 CEST 2025</t>
   </si>
 </sst>
 </file>
@@ -399,7 +417,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="27">
+  <fonts count="31">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -561,6 +579,30 @@
       <name val="Serif"/>
       <sz val="10.0"/>
       <color rgb="FFFFC800"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="15.0"/>
+      <color rgb="FFFF0000"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Courier New"/>
+      <sz val="20.0"/>
+      <color rgb="FFFF0000"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Serif"/>
+      <sz val="10.0"/>
+      <color rgb="FFFFC800"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="15.0"/>
+      <color rgb="FFFF0000"/>
       <b val="true"/>
     </font>
   </fonts>
@@ -599,7 +641,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -627,6 +669,10 @@
     <xf numFmtId="0" fontId="24" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
     <xf numFmtId="0" fontId="25" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
     <xf numFmtId="0" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
+    <xf numFmtId="0" fontId="28" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
+    <xf numFmtId="0" fontId="29" fillId="4" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
+    <xf numFmtId="0" fontId="30" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -905,17 +951,18 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="21.9375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="25.796875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="11.52734375"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="51.4921875"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="15.01171875"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="24.55859375"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="23.38671875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="25.671875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="9.703125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="32.12109375"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="19.08203125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="25.671875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="25.671875"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -923,292 +970,111 @@
         <v>0</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>116</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="23">
-        <v>28</v>
-      </c>
-      <c r="B2" t="s" s="23">
-        <v>29</v>
+      <c r="A2" t="s" s="27">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s" s="27">
+        <v>3</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>30</v>
-      </c>
-      <c r="E2" t="s" s="0">
-        <v>31</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="E2" s="0"/>
       <c r="F2" t="s" s="0">
-        <v>117</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s" s="23">
-        <v>102</v>
-      </c>
-      <c r="B3" t="s" s="23">
-        <v>103</v>
+      <c r="A3" t="s" s="27">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s" s="27">
+        <v>6</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>44</v>
+        <v>7</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>104</v>
-      </c>
-      <c r="E3" t="s" s="0">
-        <v>31</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="E3" s="0"/>
       <c r="F3" t="s" s="0">
-        <v>118</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="s" s="23">
-        <v>86</v>
-      </c>
-      <c r="B4" t="s" s="23">
-        <v>87</v>
-      </c>
-      <c r="C4" t="s" s="0">
-        <v>88</v>
-      </c>
-      <c r="D4" t="s" s="0">
-        <v>89</v>
-      </c>
-      <c r="E4" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="F4" t="s" s="0">
-        <v>117</v>
+      <c r="A4" t="s" s="0">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="s" s="23">
-        <v>62</v>
-      </c>
-      <c r="B5" t="s" s="23">
-        <v>63</v>
+      <c r="A5" t="s" s="28">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s" s="28">
+        <v>10</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>64</v>
+        <v>11</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="E5" t="s" s="0">
-        <v>66</v>
-      </c>
-      <c r="F5" t="s" s="0">
-        <v>117</v>
+        <v>12</v>
+      </c>
+      <c r="E5" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="0"/>
+      <c r="G5" t="s" s="0">
+        <v>124</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="s" s="23">
-        <v>67</v>
-      </c>
-      <c r="B6" t="s" s="23">
-        <v>63</v>
+      <c r="A6" t="s" s="29">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s" s="29">
+        <v>15</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>68</v>
+        <v>16</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>69</v>
-      </c>
-      <c r="E6" t="s" s="0">
-        <v>66</v>
-      </c>
-      <c r="F6" t="s" s="0">
-        <v>117</v>
+        <v>17</v>
+      </c>
+      <c r="E6" s="29" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="0"/>
+      <c r="G6" t="s" s="0">
+        <v>124</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="s" s="23">
-        <v>33</v>
-      </c>
-      <c r="B7" t="s" s="23">
-        <v>34</v>
+      <c r="A7" t="s" s="28">
+        <v>19</v>
+      </c>
+      <c r="B7" t="s" s="28">
+        <v>20</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>35</v>
-      </c>
-      <c r="E7" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="F7" t="s" s="0">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s" s="23">
-        <v>36</v>
-      </c>
-      <c r="B8" t="s" s="23">
-        <v>37</v>
-      </c>
-      <c r="C8" t="s" s="0">
-        <v>36</v>
-      </c>
-      <c r="D8" t="s" s="0">
-        <v>38</v>
-      </c>
-      <c r="E8" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="F8" t="s" s="0">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s" s="23">
-        <v>42</v>
-      </c>
-      <c r="B9" t="s" s="23">
-        <v>37</v>
-      </c>
-      <c r="C9" t="s" s="0">
-        <v>42</v>
-      </c>
-      <c r="D9" t="s" s="0">
-        <v>43</v>
-      </c>
-      <c r="E9" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="F9" t="s" s="0">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s" s="23">
-        <v>44</v>
-      </c>
-      <c r="B10" t="s" s="23">
-        <v>98</v>
-      </c>
-      <c r="C10" t="s" s="0">
-        <v>44</v>
-      </c>
-      <c r="D10" t="s" s="0">
-        <v>99</v>
-      </c>
-      <c r="E10" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="F10" t="s" s="0">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s" s="23">
-        <v>106</v>
-      </c>
-      <c r="B11" t="s" s="23">
-        <v>15</v>
-      </c>
-      <c r="C11" t="s" s="0">
-        <v>44</v>
-      </c>
-      <c r="D11" t="s" s="0">
-        <v>45</v>
-      </c>
-      <c r="E11" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="F11" t="s" s="0">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s" s="23">
-        <v>5</v>
-      </c>
-      <c r="B12" t="s" s="23">
-        <v>61</v>
-      </c>
-      <c r="C12" t="s" s="0">
-        <v>7</v>
-      </c>
-      <c r="D12" t="s" s="0">
-        <v>8</v>
-      </c>
-      <c r="E12" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="F12" t="s" s="0">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s" s="23">
-        <v>51</v>
-      </c>
-      <c r="B13" t="s" s="23">
-        <v>52</v>
-      </c>
-      <c r="C13" t="s" s="0">
-        <v>7</v>
-      </c>
-      <c r="D13" t="s" s="0">
-        <v>53</v>
-      </c>
-      <c r="E13" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="F13" t="s" s="0">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s" s="23">
-        <v>91</v>
-      </c>
-      <c r="B14" t="s" s="23">
-        <v>92</v>
-      </c>
-      <c r="C14" t="s" s="0">
-        <v>91</v>
-      </c>
-      <c r="D14" t="s" s="0">
-        <v>93</v>
-      </c>
-      <c r="E14" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="F14" t="s" s="0">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="s" s="23">
-        <v>46</v>
-      </c>
-      <c r="B15" t="s" s="23">
-        <v>47</v>
-      </c>
-      <c r="C15" t="s" s="0">
-        <v>7</v>
-      </c>
-      <c r="D15" t="s" s="0">
-        <v>48</v>
-      </c>
-      <c r="E15" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="F15" t="s" s="0">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="s" s="0">
-        <v>1</v>
+        <v>22</v>
+      </c>
+      <c r="E7" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="0"/>
+      <c r="G7" t="s" s="0">
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -1216,18 +1082,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="23.38671875" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="26.27734375" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="9.703125" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="32.12109375" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="26.27734375" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="19.08203125" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="26.27734375" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="21.9375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="25.671875" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="8.36328125" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="48.0703125" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="15.01171875" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="25.671875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1235,111 +1100,32 @@
         <v>0</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>120</v>
+        <v>125</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="24">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s" s="24">
-        <v>3</v>
+      <c r="A2" t="s" s="30">
+        <v>62</v>
+      </c>
+      <c r="B2" t="s" s="30">
+        <v>126</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>2</v>
+        <v>64</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="E2" s="0"/>
+        <v>65</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>66</v>
+      </c>
       <c r="F2" t="s" s="0">
-        <v>121</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s" s="24">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s" s="24">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s" s="0">
-        <v>7</v>
-      </c>
-      <c r="D3" t="s" s="0">
-        <v>8</v>
-      </c>
-      <c r="E3" s="0"/>
-      <c r="F3" t="s" s="0">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
+      <c r="A3" t="s" s="0">
         <v>1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="25">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s" s="25">
-        <v>10</v>
-      </c>
-      <c r="C5" t="s" s="0">
-        <v>11</v>
-      </c>
-      <c r="D5" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="E5" s="25" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" s="0"/>
-      <c r="G5" t="s" s="0">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="26">
-        <v>14</v>
-      </c>
-      <c r="B6" t="s" s="26">
-        <v>15</v>
-      </c>
-      <c r="C6" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="D6" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="E6" s="26" t="s">
-        <v>18</v>
-      </c>
-      <c r="F6" s="0"/>
-      <c r="G6" t="s" s="0">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s" s="25">
-        <v>19</v>
-      </c>
-      <c r="B7" t="s" s="25">
-        <v>20</v>
-      </c>
-      <c r="C7" t="s" s="0">
-        <v>21</v>
-      </c>
-      <c r="D7" t="s" s="0">
-        <v>22</v>
-      </c>
-      <c r="E7" s="25" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" s="0"/>
-      <c r="G7" t="s" s="0">
-        <v>121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Todos los test realizados. En procesao de pruebas.
</commit_message>
<xml_diff>
--- a/src/test/resources/excelTest.xlsx
+++ b/src/test/resources/excelTest.xlsx
@@ -13,8 +13,8 @@
     <workbookView xWindow="3675" yWindow="5415" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="entidadTest" r:id="rId5" sheetId="5"/>
-    <sheet name="MIT-FS.Audit4Improve-API" r:id="rId6" sheetId="6"/>
+    <sheet name="entidadTest" r:id="rId5" sheetId="7"/>
+    <sheet name="MIT-FS.Audit4Improve-API" r:id="rId6" sheetId="8"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1178" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1245" uniqueCount="138">
   <si>
     <t xml:space="preserve">Métricas guardadas el día </t>
   </si>
@@ -425,6 +425,21 @@
   </si>
   <si>
     <t>Sat May 31 12:55:13 CEST 2025</t>
+  </si>
+  <si>
+    <t>Sun Jun 01 15:52:36 CEST 2025</t>
+  </si>
+  <si>
+    <t>Sun Jun 01 13:52:36 CEST 2025</t>
+  </si>
+  <si>
+    <t>Sun Jun 01 15:52:39 CEST 2025</t>
+  </si>
+  <si>
+    <t>Sun Jun 01 15:52:37 CEST 2025</t>
+  </si>
+  <si>
+    <t>Sun Jun 01 15:52:38 CEST 2025</t>
   </si>
 </sst>
 </file>
@@ -432,7 +447,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="35">
+  <fonts count="39">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -594,6 +609,30 @@
       <name val="Serif"/>
       <sz val="10.0"/>
       <color rgb="FFFFC800"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="15.0"/>
+      <color rgb="FFFF0000"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Courier New"/>
+      <sz val="20.0"/>
+      <color rgb="FFFF0000"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Serif"/>
+      <sz val="10.0"/>
+      <color rgb="FFFFC800"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="15.0"/>
+      <color rgb="FFFF0000"/>
       <b val="true"/>
     </font>
     <font>
@@ -680,7 +719,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -716,6 +755,10 @@
     <xf numFmtId="0" fontId="32" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
     <xf numFmtId="0" fontId="33" fillId="4" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
     <xf numFmtId="0" fontId="34" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
+    <xf numFmtId="0" fontId="37" fillId="4" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
+    <xf numFmtId="0" fontId="38" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -994,18 +1037,18 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="23.38671875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="26.13671875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="25.78125"/>
     <col min="3" max="3" bestFit="true" customWidth="true" width="9.703125"/>
     <col min="4" max="4" bestFit="true" customWidth="true" width="32.12109375"/>
     <col min="5" max="5" bestFit="true" customWidth="true" width="19.08203125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="26.13671875"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="26.13671875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="25.78125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="25.78125"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1013,14 +1056,14 @@
         <v>0</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>128</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="31">
+      <c r="A2" t="s" s="35">
         <v>2</v>
       </c>
-      <c r="B2" t="s" s="31">
+      <c r="B2" t="s" s="35">
         <v>3</v>
       </c>
       <c r="C2" t="s" s="0">
@@ -1031,14 +1074,14 @@
       </c>
       <c r="E2" s="0"/>
       <c r="F2" t="s" s="0">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s" s="31">
+      <c r="A3" t="s" s="35">
         <v>5</v>
       </c>
-      <c r="B3" t="s" s="31">
+      <c r="B3" t="s" s="35">
         <v>6</v>
       </c>
       <c r="C3" t="s" s="0">
@@ -1049,7 +1092,7 @@
       </c>
       <c r="E3" s="0"/>
       <c r="F3" t="s" s="0">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4">
@@ -1058,10 +1101,10 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="s" s="32">
+      <c r="A5" t="s" s="36">
         <v>9</v>
       </c>
-      <c r="B5" t="s" s="32">
+      <c r="B5" t="s" s="36">
         <v>10</v>
       </c>
       <c r="C5" t="s" s="0">
@@ -1070,19 +1113,19 @@
       <c r="D5" t="s" s="0">
         <v>12</v>
       </c>
-      <c r="E5" s="32" t="s">
+      <c r="E5" s="36" t="s">
         <v>13</v>
       </c>
       <c r="F5" s="0"/>
       <c r="G5" t="s" s="0">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="s" s="33">
+      <c r="A6" t="s" s="37">
         <v>14</v>
       </c>
-      <c r="B6" t="s" s="33">
+      <c r="B6" t="s" s="37">
         <v>15</v>
       </c>
       <c r="C6" t="s" s="0">
@@ -1091,19 +1134,19 @@
       <c r="D6" t="s" s="0">
         <v>17</v>
       </c>
-      <c r="E6" s="33" t="s">
+      <c r="E6" s="37" t="s">
         <v>18</v>
       </c>
       <c r="F6" s="0"/>
       <c r="G6" t="s" s="0">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="s" s="32">
+      <c r="A7" t="s" s="36">
         <v>19</v>
       </c>
-      <c r="B7" t="s" s="32">
+      <c r="B7" t="s" s="36">
         <v>20</v>
       </c>
       <c r="C7" t="s" s="0">
@@ -1112,12 +1155,12 @@
       <c r="D7" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="E7" s="32" t="s">
+      <c r="E7" s="36" t="s">
         <v>13</v>
       </c>
       <c r="F7" s="0"/>
       <c r="G7" t="s" s="0">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -1125,7 +1168,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
@@ -1135,7 +1178,7 @@
     <col min="3" max="3" width="10.0" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="51.4921875" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="15.01171875" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="26.13671875" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="25.78125" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1143,14 +1186,14 @@
         <v>0</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>130</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="34">
+      <c r="A2" t="s" s="38">
         <v>5</v>
       </c>
-      <c r="B2" t="s" s="34">
+      <c r="B2" t="s" s="38">
         <v>131</v>
       </c>
       <c r="C2" t="s" s="0">
@@ -1163,14 +1206,14 @@
         <v>31</v>
       </c>
       <c r="F2" t="s" s="0">
-        <v>130</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s" s="34">
+      <c r="A3" t="s" s="38">
         <v>62</v>
       </c>
-      <c r="B3" t="s" s="34">
+      <c r="B3" t="s" s="38">
         <v>126</v>
       </c>
       <c r="C3" t="s" s="0">
@@ -1183,14 +1226,14 @@
         <v>66</v>
       </c>
       <c r="F3" t="s" s="0">
-        <v>132</v>
+        <v>136</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="s" s="34">
+      <c r="A4" t="s" s="38">
         <v>67</v>
       </c>
-      <c r="B4" t="s" s="34">
+      <c r="B4" t="s" s="38">
         <v>126</v>
       </c>
       <c r="C4" t="s" s="0">
@@ -1203,14 +1246,14 @@
         <v>66</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="s" s="34">
+      <c r="A5" t="s" s="38">
         <v>33</v>
       </c>
-      <c r="B5" t="s" s="34">
+      <c r="B5" t="s" s="38">
         <v>34</v>
       </c>
       <c r="C5" t="s" s="0">
@@ -1223,14 +1266,14 @@
         <v>31</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>130</v>
+        <v>137</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="s" s="34">
+      <c r="A6" t="s" s="38">
         <v>46</v>
       </c>
-      <c r="B6" t="s" s="34">
+      <c r="B6" t="s" s="38">
         <v>47</v>
       </c>
       <c r="C6" t="s" s="0">
@@ -1243,7 +1286,7 @@
         <v>31</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>130</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Test realizados y pasados:
</commit_message>
<xml_diff>
--- a/src/test/resources/excelTest.xlsx
+++ b/src/test/resources/excelTest.xlsx
@@ -13,8 +13,8 @@
     <workbookView xWindow="3675" yWindow="5415" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="entidadTest" r:id="rId5" sheetId="7"/>
-    <sheet name="MIT-FS.Audit4Improve-API" r:id="rId6" sheetId="8"/>
+    <sheet name="entidadTest" r:id="rId5" sheetId="11"/>
+    <sheet name="MIT-FS.Audit4Improve-API" r:id="rId6" sheetId="12"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1245" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1379" uniqueCount="147">
   <si>
     <t xml:space="preserve">Métricas guardadas el día </t>
   </si>
@@ -440,6 +440,33 @@
   </si>
   <si>
     <t>Sun Jun 01 15:52:38 CEST 2025</t>
+  </si>
+  <si>
+    <t>Sun Jun 01 17:32:57 CEST 2025</t>
+  </si>
+  <si>
+    <t>Sun Jun 01 15:32:57 CEST 2025</t>
+  </si>
+  <si>
+    <t>Sun Jun 01 17:33:00 CEST 2025</t>
+  </si>
+  <si>
+    <t>Sun Jun 01 17:32:58 CEST 2025</t>
+  </si>
+  <si>
+    <t>Sun Jun 01 17:32:59 CEST 2025</t>
+  </si>
+  <si>
+    <t>Sun Jun 01 17:44:31 CEST 2025</t>
+  </si>
+  <si>
+    <t>Sun Jun 01 15:44:31 CEST 2025</t>
+  </si>
+  <si>
+    <t>Sun Jun 01 17:44:33 CEST 2025</t>
+  </si>
+  <si>
+    <t>Sun Jun 01 17:44:32 CEST 2025</t>
   </si>
 </sst>
 </file>
@@ -447,7 +474,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="39">
+  <fonts count="47">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -609,6 +636,54 @@
       <name val="Serif"/>
       <sz val="10.0"/>
       <color rgb="FFFFC800"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="15.0"/>
+      <color rgb="FFFF0000"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Courier New"/>
+      <sz val="20.0"/>
+      <color rgb="FFFF0000"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Serif"/>
+      <sz val="10.0"/>
+      <color rgb="FFFFC800"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="15.0"/>
+      <color rgb="FFFF0000"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="15.0"/>
+      <color rgb="FFFF0000"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Courier New"/>
+      <sz val="20.0"/>
+      <color rgb="FFFF0000"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Serif"/>
+      <sz val="10.0"/>
+      <color rgb="FFFFC800"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="15.0"/>
+      <color rgb="FFFF0000"/>
       <b val="true"/>
     </font>
     <font>
@@ -719,7 +794,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -759,6 +834,14 @@
     <xf numFmtId="0" fontId="36" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
     <xf numFmtId="0" fontId="37" fillId="4" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
     <xf numFmtId="0" fontId="38" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
+    <xf numFmtId="0" fontId="39" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
+    <xf numFmtId="0" fontId="40" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
+    <xf numFmtId="0" fontId="41" fillId="4" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
+    <xf numFmtId="0" fontId="42" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
+    <xf numFmtId="0" fontId="43" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
+    <xf numFmtId="0" fontId="44" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
+    <xf numFmtId="0" fontId="45" fillId="4" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
+    <xf numFmtId="0" fontId="46" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1037,7 +1120,7 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
@@ -1056,14 +1139,14 @@
         <v>0</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>133</v>
+        <v>143</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="35">
+      <c r="A2" t="s" s="43">
         <v>2</v>
       </c>
-      <c r="B2" t="s" s="35">
+      <c r="B2" t="s" s="43">
         <v>3</v>
       </c>
       <c r="C2" t="s" s="0">
@@ -1074,14 +1157,14 @@
       </c>
       <c r="E2" s="0"/>
       <c r="F2" t="s" s="0">
-        <v>134</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s" s="35">
+      <c r="A3" t="s" s="43">
         <v>5</v>
       </c>
-      <c r="B3" t="s" s="35">
+      <c r="B3" t="s" s="43">
         <v>6</v>
       </c>
       <c r="C3" t="s" s="0">
@@ -1092,7 +1175,7 @@
       </c>
       <c r="E3" s="0"/>
       <c r="F3" t="s" s="0">
-        <v>134</v>
+        <v>144</v>
       </c>
     </row>
     <row r="4">
@@ -1101,10 +1184,10 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="s" s="36">
+      <c r="A5" t="s" s="44">
         <v>9</v>
       </c>
-      <c r="B5" t="s" s="36">
+      <c r="B5" t="s" s="44">
         <v>10</v>
       </c>
       <c r="C5" t="s" s="0">
@@ -1113,19 +1196,19 @@
       <c r="D5" t="s" s="0">
         <v>12</v>
       </c>
-      <c r="E5" s="36" t="s">
+      <c r="E5" s="44" t="s">
         <v>13</v>
       </c>
       <c r="F5" s="0"/>
       <c r="G5" t="s" s="0">
-        <v>134</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="s" s="37">
+      <c r="A6" t="s" s="45">
         <v>14</v>
       </c>
-      <c r="B6" t="s" s="37">
+      <c r="B6" t="s" s="45">
         <v>15</v>
       </c>
       <c r="C6" t="s" s="0">
@@ -1134,19 +1217,19 @@
       <c r="D6" t="s" s="0">
         <v>17</v>
       </c>
-      <c r="E6" s="37" t="s">
+      <c r="E6" s="45" t="s">
         <v>18</v>
       </c>
       <c r="F6" s="0"/>
       <c r="G6" t="s" s="0">
-        <v>134</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="s" s="36">
+      <c r="A7" t="s" s="44">
         <v>19</v>
       </c>
-      <c r="B7" t="s" s="36">
+      <c r="B7" t="s" s="44">
         <v>20</v>
       </c>
       <c r="C7" t="s" s="0">
@@ -1155,12 +1238,12 @@
       <c r="D7" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="E7" s="36" t="s">
+      <c r="E7" s="44" t="s">
         <v>13</v>
       </c>
       <c r="F7" s="0"/>
       <c r="G7" t="s" s="0">
-        <v>134</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -1168,7 +1251,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
@@ -1186,14 +1269,14 @@
         <v>0</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>135</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="38">
+      <c r="A2" t="s" s="46">
         <v>5</v>
       </c>
-      <c r="B2" t="s" s="38">
+      <c r="B2" t="s" s="46">
         <v>131</v>
       </c>
       <c r="C2" t="s" s="0">
@@ -1206,14 +1289,14 @@
         <v>31</v>
       </c>
       <c r="F2" t="s" s="0">
-        <v>135</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s" s="38">
+      <c r="A3" t="s" s="46">
         <v>62</v>
       </c>
-      <c r="B3" t="s" s="38">
+      <c r="B3" t="s" s="46">
         <v>126</v>
       </c>
       <c r="C3" t="s" s="0">
@@ -1226,14 +1309,14 @@
         <v>66</v>
       </c>
       <c r="F3" t="s" s="0">
-        <v>136</v>
+        <v>146</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="s" s="38">
+      <c r="A4" t="s" s="46">
         <v>67</v>
       </c>
-      <c r="B4" t="s" s="38">
+      <c r="B4" t="s" s="46">
         <v>126</v>
       </c>
       <c r="C4" t="s" s="0">
@@ -1246,14 +1329,14 @@
         <v>66</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>137</v>
+        <v>146</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="s" s="38">
+      <c r="A5" t="s" s="46">
         <v>33</v>
       </c>
-      <c r="B5" t="s" s="38">
+      <c r="B5" t="s" s="46">
         <v>34</v>
       </c>
       <c r="C5" t="s" s="0">
@@ -1266,14 +1349,14 @@
         <v>31</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>137</v>
+        <v>146</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="s" s="38">
+      <c r="A6" t="s" s="46">
         <v>46</v>
       </c>
-      <c r="B6" t="s" s="38">
+      <c r="B6" t="s" s="46">
         <v>47</v>
       </c>
       <c r="C6" t="s" s="0">
@@ -1286,7 +1369,7 @@
         <v>31</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>137</v>
+        <v>145</v>
       </c>
     </row>
     <row r="7">

</xml_diff>